<commit_message>
add name and title for ruim 7f3df81c7fa5db662fce40fb57532dce7a5ed33c
</commit_message>
<xml_diff>
--- a/nriss-patch-1/ig/StructureDefinition-profile-ruim-codesystem.xlsx
+++ b/nriss-patch-1/ig/StructureDefinition-profile-ruim-codesystem.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4246" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4246" uniqueCount="473">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-27T13:12:34+00:00</t>
+    <t>2026-03-27T13:20:16+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -547,6 +547,9 @@
     <t>Support human navigation and code generation.</t>
   </si>
   <si>
+    <t>RUIM eeprescription</t>
+  </si>
+  <si>
     <t xml:space="preserve">inv-0
 </t>
   </si>
@@ -561,6 +564,9 @@
   </si>
   <si>
     <t>This name does not need to be machine-processing friendly and may contain punctuation, white-space, etc.</t>
+  </si>
+  <si>
+    <t>RUIM - european eprescription</t>
   </si>
   <si>
     <t>Definition.title</t>
@@ -3372,7 +3378,7 @@
         <v>77</v>
       </c>
       <c r="S14" t="s" s="2">
-        <v>77</v>
+        <v>170</v>
       </c>
       <c r="T14" t="s" s="2">
         <v>77</v>
@@ -3420,7 +3426,7 @@
         <v>78</v>
       </c>
       <c r="AI14" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AJ14" t="s" s="2">
         <v>98</v>
@@ -3440,10 +3446,10 @@
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -3451,7 +3457,7 @@
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G15" t="s" s="2">
         <v>78</v>
@@ -3469,13 +3475,13 @@
         <v>159</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="N15" t="s" s="2">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">
@@ -3486,7 +3492,7 @@
         <v>77</v>
       </c>
       <c r="S15" t="s" s="2">
-        <v>77</v>
+        <v>176</v>
       </c>
       <c r="T15" t="s" s="2">
         <v>77</v>
@@ -3525,7 +3531,7 @@
         <v>77</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>82</v>
@@ -3543,7 +3549,7 @@
         <v>77</v>
       </c>
       <c r="AL15" t="s" s="2">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AM15" t="s" s="2">
         <v>77</v>
@@ -3554,10 +3560,10 @@
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -3583,13 +3589,13 @@
         <v>106</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="N16" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="O16" s="2"/>
       <c r="P16" t="s" s="2">
@@ -3615,13 +3621,13 @@
         <v>77</v>
       </c>
       <c r="X16" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Y16" t="s" s="2">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="Z16" t="s" s="2">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="AA16" t="s" s="2">
         <v>77</v>
@@ -3639,7 +3645,7 @@
         <v>77</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>78</v>
@@ -3657,10 +3663,10 @@
         <v>85</v>
       </c>
       <c r="AL16" t="s" s="2">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="AM16" t="s" s="2">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="AN16" t="s" s="2">
         <v>77</v>
@@ -3668,10 +3674,10 @@
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3694,19 +3700,19 @@
         <v>87</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="N17" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="O17" t="s" s="2">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="P17" t="s" s="2">
         <v>77</v>
@@ -3755,7 +3761,7 @@
         <v>77</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>82</v>
@@ -3773,10 +3779,10 @@
         <v>77</v>
       </c>
       <c r="AL17" t="s" s="2">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="AM17" t="s" s="2">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="AN17" t="s" s="2">
         <v>77</v>
@@ -3784,14 +3790,14 @@
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
@@ -3810,16 +3816,16 @@
         <v>87</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -3869,7 +3875,7 @@
         <v>77</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>82</v>
@@ -3887,10 +3893,10 @@
         <v>77</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="AM18" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="AN18" t="s" s="2">
         <v>77</v>
@@ -3898,14 +3904,14 @@
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
@@ -3927,16 +3933,16 @@
         <v>159</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="O19" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="P19" t="s" s="2">
         <v>77</v>
@@ -3985,7 +3991,7 @@
         <v>77</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>82</v>
@@ -4003,10 +4009,10 @@
         <v>77</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="AM19" t="s" s="2">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="AN19" t="s" s="2">
         <v>77</v>
@@ -4014,10 +4020,10 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -4040,16 +4046,16 @@
         <v>87</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="N20" t="s" s="2">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
@@ -4099,7 +4105,7 @@
         <v>77</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>82</v>
@@ -4117,7 +4123,7 @@
         <v>77</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="AM20" t="s" s="2">
         <v>77</v>
@@ -4128,14 +4134,14 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" t="s" s="2">
@@ -4154,16 +4160,16 @@
         <v>77</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="N21" t="s" s="2">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
@@ -4213,7 +4219,7 @@
         <v>77</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>82</v>
@@ -4231,7 +4237,7 @@
         <v>85</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="AM21" t="s" s="2">
         <v>77</v>
@@ -4242,10 +4248,10 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4268,19 +4274,19 @@
         <v>87</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="N22" t="s" s="2">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="O22" t="s" s="2">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="P22" t="s" s="2">
         <v>77</v>
@@ -4329,7 +4335,7 @@
         <v>77</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>82</v>
@@ -4347,7 +4353,7 @@
         <v>77</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="AM22" t="s" s="2">
         <v>77</v>
@@ -4358,10 +4364,10 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -4384,16 +4390,16 @@
         <v>87</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -4419,13 +4425,13 @@
         <v>77</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Y23" t="s" s="2">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="Z23" t="s" s="2">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>77</v>
@@ -4443,7 +4449,7 @@
         <v>77</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>82</v>
@@ -4461,7 +4467,7 @@
         <v>77</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="AM23" t="s" s="2">
         <v>77</v>
@@ -4472,10 +4478,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4498,16 +4504,16 @@
         <v>77</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="O24" s="2"/>
       <c r="P24" t="s" s="2">
@@ -4557,7 +4563,7 @@
         <v>77</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>82</v>
@@ -4575,10 +4581,10 @@
         <v>77</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="AN24" t="s" s="2">
         <v>157</v>
@@ -4586,14 +4592,14 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
@@ -4612,19 +4618,19 @@
         <v>77</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="O25" t="s" s="2">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>77</v>
@@ -4673,7 +4679,7 @@
         <v>77</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>82</v>
@@ -4691,7 +4697,7 @@
         <v>77</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="AM25" t="s" s="2">
         <v>77</v>
@@ -4702,10 +4708,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4728,16 +4734,16 @@
         <v>87</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
@@ -4787,7 +4793,7 @@
         <v>77</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>82</v>
@@ -4816,10 +4822,10 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4842,16 +4848,16 @@
         <v>87</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="N27" t="s" s="2">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
@@ -4901,7 +4907,7 @@
         <v>77</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>82</v>
@@ -4930,10 +4936,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4959,13 +4965,13 @@
         <v>106</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -4991,13 +4997,13 @@
         <v>77</v>
       </c>
       <c r="X28" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Y28" t="s" s="2">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="Z28" t="s" s="2">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="AA28" t="s" s="2">
         <v>77</v>
@@ -5015,7 +5021,7 @@
         <v>77</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>82</v>
@@ -5044,14 +5050,14 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
@@ -5070,16 +5076,16 @@
         <v>87</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
@@ -5129,7 +5135,7 @@
         <v>77</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>82</v>
@@ -5158,10 +5164,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5184,16 +5190,16 @@
         <v>87</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
@@ -5243,7 +5249,7 @@
         <v>77</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>82</v>
@@ -5272,10 +5278,10 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5301,10 +5307,10 @@
         <v>106</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -5331,13 +5337,13 @@
         <v>77</v>
       </c>
       <c r="X31" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Y31" t="s" s="2">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="Z31" t="s" s="2">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="AA31" t="s" s="2">
         <v>77</v>
@@ -5355,7 +5361,7 @@
         <v>77</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
@@ -5384,10 +5390,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5410,16 +5416,16 @@
         <v>87</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
@@ -5469,7 +5475,7 @@
         <v>77</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>82</v>
@@ -5498,10 +5504,10 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5524,16 +5530,16 @@
         <v>87</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -5583,7 +5589,7 @@
         <v>77</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>82</v>
@@ -5612,10 +5618,10 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5638,16 +5644,16 @@
         <v>87</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
@@ -5697,7 +5703,7 @@
         <v>77</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>82</v>
@@ -5726,10 +5732,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5755,10 +5761,10 @@
         <v>159</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -5809,7 +5815,7 @@
         <v>77</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>82</v>
@@ -5824,7 +5830,7 @@
         <v>77</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>77</v>
@@ -5838,10 +5844,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5870,7 +5876,7 @@
         <v>132</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N36" t="s" s="2">
         <v>134</v>
@@ -5923,7 +5929,7 @@
         <v>77</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>82</v>
@@ -5938,7 +5944,7 @@
         <v>136</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>77</v>
@@ -5952,14 +5958,14 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
@@ -5981,10 +5987,10 @@
         <v>131</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N37" t="s" s="2">
         <v>134</v>
@@ -6039,7 +6045,7 @@
         <v>77</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>82</v>
@@ -6068,10 +6074,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6097,10 +6103,10 @@
         <v>106</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -6151,7 +6157,7 @@
         <v>77</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
@@ -6180,10 +6186,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6209,10 +6215,10 @@
         <v>159</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -6263,7 +6269,7 @@
         <v>77</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>82</v>
@@ -6292,10 +6298,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6321,10 +6327,10 @@
         <v>106</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -6351,13 +6357,13 @@
         <v>77</v>
       </c>
       <c r="X40" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Y40" t="s" s="2">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="Z40" t="s" s="2">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="AA40" t="s" s="2">
         <v>77</v>
@@ -6375,7 +6381,7 @@
         <v>77</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
@@ -6404,10 +6410,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6433,10 +6439,10 @@
         <v>159</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -6487,7 +6493,7 @@
         <v>77</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
@@ -6516,10 +6522,10 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6542,13 +6548,13 @@
         <v>87</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6587,17 +6593,17 @@
         <v>77</v>
       </c>
       <c r="AB42" t="s" s="2">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="AC42" s="2"/>
       <c r="AD42" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE42" t="s" s="2">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>82</v>
@@ -6626,10 +6632,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6655,10 +6661,10 @@
         <v>159</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -6709,7 +6715,7 @@
         <v>77</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>82</v>
@@ -6724,7 +6730,7 @@
         <v>77</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL43" t="s" s="2">
         <v>77</v>
@@ -6738,10 +6744,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6770,7 +6776,7 @@
         <v>132</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N44" t="s" s="2">
         <v>134</v>
@@ -6823,7 +6829,7 @@
         <v>77</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>82</v>
@@ -6838,7 +6844,7 @@
         <v>136</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>77</v>
@@ -6852,14 +6858,14 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
@@ -6881,10 +6887,10 @@
         <v>131</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N45" t="s" s="2">
         <v>134</v>
@@ -6939,7 +6945,7 @@
         <v>77</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>82</v>
@@ -6968,10 +6974,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6997,10 +7003,10 @@
         <v>106</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -7027,11 +7033,11 @@
         <v>77</v>
       </c>
       <c r="X46" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Y46" s="2"/>
       <c r="Z46" t="s" s="2">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>77</v>
@@ -7049,7 +7055,7 @@
         <v>77</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>78</v>
@@ -7078,10 +7084,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7107,10 +7113,10 @@
         <v>100</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -7161,7 +7167,7 @@
         <v>77</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>82</v>
@@ -7190,10 +7196,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7219,10 +7225,10 @@
         <v>159</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -7273,7 +7279,7 @@
         <v>77</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>82</v>
@@ -7302,10 +7308,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7331,10 +7337,10 @@
         <v>106</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
@@ -7361,13 +7367,13 @@
         <v>77</v>
       </c>
       <c r="X49" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Y49" t="s" s="2">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="Z49" t="s" s="2">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="AA49" t="s" s="2">
         <v>77</v>
@@ -7385,7 +7391,7 @@
         <v>77</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>78</v>
@@ -7414,13 +7420,13 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C50" t="s" s="2">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="D50" t="s" s="2">
         <v>77</v>
@@ -7442,13 +7448,13 @@
         <v>87</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -7499,7 +7505,7 @@
         <v>77</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>82</v>
@@ -7528,10 +7534,10 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7557,10 +7563,10 @@
         <v>159</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
@@ -7611,7 +7617,7 @@
         <v>77</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>82</v>
@@ -7626,7 +7632,7 @@
         <v>77</v>
       </c>
       <c r="AK51" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL51" t="s" s="2">
         <v>77</v>
@@ -7640,10 +7646,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -7672,7 +7678,7 @@
         <v>132</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N52" t="s" s="2">
         <v>134</v>
@@ -7725,7 +7731,7 @@
         <v>77</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>82</v>
@@ -7740,7 +7746,7 @@
         <v>136</v>
       </c>
       <c r="AK52" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL52" t="s" s="2">
         <v>77</v>
@@ -7754,14 +7760,14 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E53" s="2"/>
       <c r="F53" t="s" s="2">
@@ -7783,10 +7789,10 @@
         <v>131</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N53" t="s" s="2">
         <v>134</v>
@@ -7841,7 +7847,7 @@
         <v>77</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>82</v>
@@ -7870,10 +7876,10 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -7899,10 +7905,10 @@
         <v>106</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -7914,7 +7920,7 @@
         <v>77</v>
       </c>
       <c r="S54" t="s" s="2">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="T54" t="s" s="2">
         <v>77</v>
@@ -7929,11 +7935,11 @@
         <v>77</v>
       </c>
       <c r="X54" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Y54" s="2"/>
       <c r="Z54" t="s" s="2">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>77</v>
@@ -7951,7 +7957,7 @@
         <v>77</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>78</v>
@@ -7980,10 +7986,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8009,10 +8015,10 @@
         <v>100</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -8024,7 +8030,7 @@
         <v>77</v>
       </c>
       <c r="S55" t="s" s="2">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="T55" t="s" s="2">
         <v>77</v>
@@ -8063,7 +8069,7 @@
         <v>77</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>82</v>
@@ -8092,10 +8098,10 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8121,10 +8127,10 @@
         <v>159</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
@@ -8175,7 +8181,7 @@
         <v>77</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>82</v>
@@ -8204,10 +8210,10 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8233,10 +8239,10 @@
         <v>106</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
@@ -8248,7 +8254,7 @@
         <v>77</v>
       </c>
       <c r="S57" t="s" s="2">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="T57" t="s" s="2">
         <v>77</v>
@@ -8263,13 +8269,13 @@
         <v>77</v>
       </c>
       <c r="X57" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Y57" t="s" s="2">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="Z57" t="s" s="2">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="AA57" t="s" s="2">
         <v>77</v>
@@ -8287,7 +8293,7 @@
         <v>77</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>78</v>
@@ -8316,13 +8322,13 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C58" t="s" s="2">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="D58" t="s" s="2">
         <v>77</v>
@@ -8344,13 +8350,13 @@
         <v>87</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -8401,7 +8407,7 @@
         <v>77</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>82</v>
@@ -8430,10 +8436,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -8459,10 +8465,10 @@
         <v>159</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
@@ -8513,7 +8519,7 @@
         <v>77</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>82</v>
@@ -8528,7 +8534,7 @@
         <v>77</v>
       </c>
       <c r="AK59" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL59" t="s" s="2">
         <v>77</v>
@@ -8542,10 +8548,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -8574,7 +8580,7 @@
         <v>132</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N60" t="s" s="2">
         <v>134</v>
@@ -8627,7 +8633,7 @@
         <v>77</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>82</v>
@@ -8642,7 +8648,7 @@
         <v>136</v>
       </c>
       <c r="AK60" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL60" t="s" s="2">
         <v>77</v>
@@ -8656,14 +8662,14 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E61" s="2"/>
       <c r="F61" t="s" s="2">
@@ -8685,10 +8691,10 @@
         <v>131</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N61" t="s" s="2">
         <v>134</v>
@@ -8743,7 +8749,7 @@
         <v>77</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>82</v>
@@ -8772,10 +8778,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -8801,10 +8807,10 @@
         <v>106</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -8816,7 +8822,7 @@
         <v>77</v>
       </c>
       <c r="S62" t="s" s="2">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="T62" t="s" s="2">
         <v>77</v>
@@ -8831,11 +8837,11 @@
         <v>77</v>
       </c>
       <c r="X62" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Y62" s="2"/>
       <c r="Z62" t="s" s="2">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="AA62" t="s" s="2">
         <v>77</v>
@@ -8853,7 +8859,7 @@
         <v>77</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>78</v>
@@ -8882,10 +8888,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -8911,10 +8917,10 @@
         <v>100</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
@@ -8926,7 +8932,7 @@
         <v>77</v>
       </c>
       <c r="S63" t="s" s="2">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="T63" t="s" s="2">
         <v>77</v>
@@ -8965,7 +8971,7 @@
         <v>77</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>82</v>
@@ -8994,10 +9000,10 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9023,10 +9029,10 @@
         <v>159</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
@@ -9077,7 +9083,7 @@
         <v>77</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>82</v>
@@ -9106,10 +9112,10 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -9135,10 +9141,10 @@
         <v>106</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
@@ -9150,7 +9156,7 @@
         <v>77</v>
       </c>
       <c r="S65" t="s" s="2">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="T65" t="s" s="2">
         <v>77</v>
@@ -9165,13 +9171,13 @@
         <v>77</v>
       </c>
       <c r="X65" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Y65" t="s" s="2">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="Z65" t="s" s="2">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="AA65" t="s" s="2">
         <v>77</v>
@@ -9189,7 +9195,7 @@
         <v>77</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>78</v>
@@ -9218,13 +9224,13 @@
     </row>
     <row r="66">
       <c r="A66" t="s" s="2">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C66" t="s" s="2">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D66" t="s" s="2">
         <v>77</v>
@@ -9246,13 +9252,13 @@
         <v>87</v>
       </c>
       <c r="K66" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L66" t="s" s="2">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="M66" t="s" s="2">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
@@ -9303,7 +9309,7 @@
         <v>77</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>82</v>
@@ -9332,10 +9338,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -9361,10 +9367,10 @@
         <v>159</v>
       </c>
       <c r="L67" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="M67" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N67" s="2"/>
       <c r="O67" s="2"/>
@@ -9415,7 +9421,7 @@
         <v>77</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>82</v>
@@ -9430,7 +9436,7 @@
         <v>77</v>
       </c>
       <c r="AK67" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL67" t="s" s="2">
         <v>77</v>
@@ -9444,10 +9450,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -9476,7 +9482,7 @@
         <v>132</v>
       </c>
       <c r="M68" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N68" t="s" s="2">
         <v>134</v>
@@ -9529,7 +9535,7 @@
         <v>77</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>82</v>
@@ -9544,7 +9550,7 @@
         <v>136</v>
       </c>
       <c r="AK68" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL68" t="s" s="2">
         <v>77</v>
@@ -9558,14 +9564,14 @@
     </row>
     <row r="69" hidden="true">
       <c r="A69" t="s" s="2">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E69" s="2"/>
       <c r="F69" t="s" s="2">
@@ -9587,10 +9593,10 @@
         <v>131</v>
       </c>
       <c r="L69" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M69" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N69" t="s" s="2">
         <v>134</v>
@@ -9645,7 +9651,7 @@
         <v>77</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>82</v>
@@ -9674,10 +9680,10 @@
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -9703,10 +9709,10 @@
         <v>106</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="N70" s="2"/>
       <c r="O70" s="2"/>
@@ -9718,7 +9724,7 @@
         <v>77</v>
       </c>
       <c r="S70" t="s" s="2">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="T70" t="s" s="2">
         <v>77</v>
@@ -9733,11 +9739,11 @@
         <v>77</v>
       </c>
       <c r="X70" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Y70" s="2"/>
       <c r="Z70" t="s" s="2">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="AA70" t="s" s="2">
         <v>77</v>
@@ -9755,7 +9761,7 @@
         <v>77</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>78</v>
@@ -9784,10 +9790,10 @@
     </row>
     <row r="71" hidden="true">
       <c r="A71" t="s" s="2">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -9813,10 +9819,10 @@
         <v>100</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
@@ -9828,7 +9834,7 @@
         <v>77</v>
       </c>
       <c r="S71" t="s" s="2">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="T71" t="s" s="2">
         <v>77</v>
@@ -9867,7 +9873,7 @@
         <v>77</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>82</v>
@@ -9896,10 +9902,10 @@
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -9925,10 +9931,10 @@
         <v>159</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
@@ -9979,7 +9985,7 @@
         <v>77</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>82</v>
@@ -10008,10 +10014,10 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -10037,10 +10043,10 @@
         <v>106</v>
       </c>
       <c r="L73" t="s" s="2">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="M73" t="s" s="2">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="N73" s="2"/>
       <c r="O73" s="2"/>
@@ -10052,7 +10058,7 @@
         <v>77</v>
       </c>
       <c r="S73" t="s" s="2">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="T73" t="s" s="2">
         <v>77</v>
@@ -10067,13 +10073,13 @@
         <v>77</v>
       </c>
       <c r="X73" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Y73" t="s" s="2">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="Z73" t="s" s="2">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="AA73" t="s" s="2">
         <v>77</v>
@@ -10091,7 +10097,7 @@
         <v>77</v>
       </c>
       <c r="AF73" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="AG73" t="s" s="2">
         <v>78</v>
@@ -10120,13 +10126,13 @@
     </row>
     <row r="74">
       <c r="A74" t="s" s="2">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C74" t="s" s="2">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D74" t="s" s="2">
         <v>77</v>
@@ -10148,13 +10154,13 @@
         <v>87</v>
       </c>
       <c r="K74" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L74" t="s" s="2">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="M74" t="s" s="2">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="N74" s="2"/>
       <c r="O74" s="2"/>
@@ -10205,7 +10211,7 @@
         <v>77</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>82</v>
@@ -10234,10 +10240,10 @@
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -10263,10 +10269,10 @@
         <v>159</v>
       </c>
       <c r="L75" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="M75" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
@@ -10317,7 +10323,7 @@
         <v>77</v>
       </c>
       <c r="AF75" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>82</v>
@@ -10332,7 +10338,7 @@
         <v>77</v>
       </c>
       <c r="AK75" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL75" t="s" s="2">
         <v>77</v>
@@ -10346,10 +10352,10 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -10378,7 +10384,7 @@
         <v>132</v>
       </c>
       <c r="M76" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N76" t="s" s="2">
         <v>134</v>
@@ -10431,7 +10437,7 @@
         <v>77</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>82</v>
@@ -10446,7 +10452,7 @@
         <v>136</v>
       </c>
       <c r="AK76" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL76" t="s" s="2">
         <v>77</v>
@@ -10460,14 +10466,14 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E77" s="2"/>
       <c r="F77" t="s" s="2">
@@ -10489,10 +10495,10 @@
         <v>131</v>
       </c>
       <c r="L77" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M77" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N77" t="s" s="2">
         <v>134</v>
@@ -10547,7 +10553,7 @@
         <v>77</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>82</v>
@@ -10576,10 +10582,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -10605,10 +10611,10 @@
         <v>106</v>
       </c>
       <c r="L78" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="M78" t="s" s="2">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="N78" s="2"/>
       <c r="O78" s="2"/>
@@ -10620,7 +10626,7 @@
         <v>77</v>
       </c>
       <c r="S78" t="s" s="2">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="T78" t="s" s="2">
         <v>77</v>
@@ -10635,11 +10641,11 @@
         <v>77</v>
       </c>
       <c r="X78" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Y78" s="2"/>
       <c r="Z78" t="s" s="2">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="AA78" t="s" s="2">
         <v>77</v>
@@ -10657,7 +10663,7 @@
         <v>77</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>78</v>
@@ -10686,10 +10692,10 @@
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -10715,10 +10721,10 @@
         <v>100</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="M79" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="N79" s="2"/>
       <c r="O79" s="2"/>
@@ -10730,7 +10736,7 @@
         <v>77</v>
       </c>
       <c r="S79" t="s" s="2">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="T79" t="s" s="2">
         <v>77</v>
@@ -10769,7 +10775,7 @@
         <v>77</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>82</v>
@@ -10798,10 +10804,10 @@
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -10827,10 +10833,10 @@
         <v>159</v>
       </c>
       <c r="L80" t="s" s="2">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="M80" t="s" s="2">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="N80" s="2"/>
       <c r="O80" s="2"/>
@@ -10881,7 +10887,7 @@
         <v>77</v>
       </c>
       <c r="AF80" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="AG80" t="s" s="2">
         <v>82</v>
@@ -10910,10 +10916,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -10939,10 +10945,10 @@
         <v>106</v>
       </c>
       <c r="L81" t="s" s="2">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="M81" t="s" s="2">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="N81" s="2"/>
       <c r="O81" s="2"/>
@@ -10954,7 +10960,7 @@
         <v>77</v>
       </c>
       <c r="S81" t="s" s="2">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="T81" t="s" s="2">
         <v>77</v>
@@ -10969,13 +10975,13 @@
         <v>77</v>
       </c>
       <c r="X81" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Y81" t="s" s="2">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="Z81" t="s" s="2">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="AA81" t="s" s="2">
         <v>77</v>
@@ -10993,7 +10999,7 @@
         <v>77</v>
       </c>
       <c r="AF81" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="AG81" t="s" s="2">
         <v>78</v>
@@ -11022,13 +11028,13 @@
     </row>
     <row r="82">
       <c r="A82" t="s" s="2">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C82" t="s" s="2">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D82" t="s" s="2">
         <v>77</v>
@@ -11050,13 +11056,13 @@
         <v>87</v>
       </c>
       <c r="K82" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L82" t="s" s="2">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="M82" t="s" s="2">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="N82" s="2"/>
       <c r="O82" s="2"/>
@@ -11107,7 +11113,7 @@
         <v>77</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>82</v>
@@ -11136,10 +11142,10 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -11165,10 +11171,10 @@
         <v>159</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N83" s="2"/>
       <c r="O83" s="2"/>
@@ -11219,7 +11225,7 @@
         <v>77</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>82</v>
@@ -11234,7 +11240,7 @@
         <v>77</v>
       </c>
       <c r="AK83" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL83" t="s" s="2">
         <v>77</v>
@@ -11248,10 +11254,10 @@
     </row>
     <row r="84" hidden="true">
       <c r="A84" t="s" s="2">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -11280,7 +11286,7 @@
         <v>132</v>
       </c>
       <c r="M84" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N84" t="s" s="2">
         <v>134</v>
@@ -11333,7 +11339,7 @@
         <v>77</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>82</v>
@@ -11348,7 +11354,7 @@
         <v>136</v>
       </c>
       <c r="AK84" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL84" t="s" s="2">
         <v>77</v>
@@ -11362,14 +11368,14 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E85" s="2"/>
       <c r="F85" t="s" s="2">
@@ -11391,10 +11397,10 @@
         <v>131</v>
       </c>
       <c r="L85" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M85" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N85" t="s" s="2">
         <v>134</v>
@@ -11449,7 +11455,7 @@
         <v>77</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>82</v>
@@ -11478,10 +11484,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -11507,10 +11513,10 @@
         <v>106</v>
       </c>
       <c r="L86" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="M86" t="s" s="2">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="N86" s="2"/>
       <c r="O86" s="2"/>
@@ -11522,7 +11528,7 @@
         <v>77</v>
       </c>
       <c r="S86" t="s" s="2">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="T86" t="s" s="2">
         <v>77</v>
@@ -11537,11 +11543,11 @@
         <v>77</v>
       </c>
       <c r="X86" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Y86" s="2"/>
       <c r="Z86" t="s" s="2">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="AA86" t="s" s="2">
         <v>77</v>
@@ -11559,7 +11565,7 @@
         <v>77</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>78</v>
@@ -11588,10 +11594,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -11617,10 +11623,10 @@
         <v>100</v>
       </c>
       <c r="L87" t="s" s="2">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="M87" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="N87" s="2"/>
       <c r="O87" s="2"/>
@@ -11632,7 +11638,7 @@
         <v>77</v>
       </c>
       <c r="S87" t="s" s="2">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="T87" t="s" s="2">
         <v>77</v>
@@ -11671,7 +11677,7 @@
         <v>77</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>82</v>
@@ -11700,10 +11706,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -11729,10 +11735,10 @@
         <v>159</v>
       </c>
       <c r="L88" t="s" s="2">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="M88" t="s" s="2">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="N88" s="2"/>
       <c r="O88" s="2"/>
@@ -11783,7 +11789,7 @@
         <v>77</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>82</v>
@@ -11812,10 +11818,10 @@
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -11841,10 +11847,10 @@
         <v>106</v>
       </c>
       <c r="L89" t="s" s="2">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="M89" t="s" s="2">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="N89" s="2"/>
       <c r="O89" s="2"/>
@@ -11856,7 +11862,7 @@
         <v>77</v>
       </c>
       <c r="S89" t="s" s="2">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="T89" t="s" s="2">
         <v>77</v>
@@ -11871,13 +11877,13 @@
         <v>77</v>
       </c>
       <c r="X89" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Y89" t="s" s="2">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="Z89" t="s" s="2">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="AA89" t="s" s="2">
         <v>77</v>
@@ -11895,7 +11901,7 @@
         <v>77</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>78</v>
@@ -11924,13 +11930,13 @@
     </row>
     <row r="90">
       <c r="A90" t="s" s="2">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C90" t="s" s="2">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D90" t="s" s="2">
         <v>77</v>
@@ -11952,13 +11958,13 @@
         <v>87</v>
       </c>
       <c r="K90" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L90" t="s" s="2">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="M90" t="s" s="2">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="N90" s="2"/>
       <c r="O90" s="2"/>
@@ -12009,7 +12015,7 @@
         <v>77</v>
       </c>
       <c r="AF90" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="AG90" t="s" s="2">
         <v>82</v>
@@ -12038,10 +12044,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -12067,10 +12073,10 @@
         <v>159</v>
       </c>
       <c r="L91" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="M91" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N91" s="2"/>
       <c r="O91" s="2"/>
@@ -12121,7 +12127,7 @@
         <v>77</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>82</v>
@@ -12136,7 +12142,7 @@
         <v>77</v>
       </c>
       <c r="AK91" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL91" t="s" s="2">
         <v>77</v>
@@ -12150,10 +12156,10 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -12182,7 +12188,7 @@
         <v>132</v>
       </c>
       <c r="M92" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N92" t="s" s="2">
         <v>134</v>
@@ -12235,7 +12241,7 @@
         <v>77</v>
       </c>
       <c r="AF92" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="AG92" t="s" s="2">
         <v>82</v>
@@ -12250,7 +12256,7 @@
         <v>136</v>
       </c>
       <c r="AK92" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL92" t="s" s="2">
         <v>77</v>
@@ -12264,14 +12270,14 @@
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E93" s="2"/>
       <c r="F93" t="s" s="2">
@@ -12293,10 +12299,10 @@
         <v>131</v>
       </c>
       <c r="L93" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M93" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N93" t="s" s="2">
         <v>134</v>
@@ -12351,7 +12357,7 @@
         <v>77</v>
       </c>
       <c r="AF93" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AG93" t="s" s="2">
         <v>82</v>
@@ -12380,10 +12386,10 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -12409,10 +12415,10 @@
         <v>106</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="N94" s="2"/>
       <c r="O94" s="2"/>
@@ -12424,7 +12430,7 @@
         <v>77</v>
       </c>
       <c r="S94" t="s" s="2">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="T94" t="s" s="2">
         <v>77</v>
@@ -12439,11 +12445,11 @@
         <v>77</v>
       </c>
       <c r="X94" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Y94" s="2"/>
       <c r="Z94" t="s" s="2">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="AA94" t="s" s="2">
         <v>77</v>
@@ -12461,7 +12467,7 @@
         <v>77</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>78</v>
@@ -12490,10 +12496,10 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -12519,10 +12525,10 @@
         <v>100</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="N95" s="2"/>
       <c r="O95" s="2"/>
@@ -12534,7 +12540,7 @@
         <v>77</v>
       </c>
       <c r="S95" t="s" s="2">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="T95" t="s" s="2">
         <v>77</v>
@@ -12573,7 +12579,7 @@
         <v>77</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>82</v>
@@ -12602,10 +12608,10 @@
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -12631,10 +12637,10 @@
         <v>159</v>
       </c>
       <c r="L96" t="s" s="2">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="M96" t="s" s="2">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="N96" s="2"/>
       <c r="O96" s="2"/>
@@ -12685,7 +12691,7 @@
         <v>77</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>82</v>
@@ -12714,10 +12720,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -12743,10 +12749,10 @@
         <v>106</v>
       </c>
       <c r="L97" t="s" s="2">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="M97" t="s" s="2">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="N97" s="2"/>
       <c r="O97" s="2"/>
@@ -12758,7 +12764,7 @@
         <v>77</v>
       </c>
       <c r="S97" t="s" s="2">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="T97" t="s" s="2">
         <v>77</v>
@@ -12773,13 +12779,13 @@
         <v>77</v>
       </c>
       <c r="X97" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Y97" t="s" s="2">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="Z97" t="s" s="2">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="AA97" t="s" s="2">
         <v>77</v>
@@ -12797,7 +12803,7 @@
         <v>77</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>78</v>
@@ -12826,10 +12832,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -12852,16 +12858,16 @@
         <v>77</v>
       </c>
       <c r="K98" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L98" t="s" s="2">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="M98" t="s" s="2">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="N98" t="s" s="2">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="O98" s="2"/>
       <c r="P98" t="s" s="2">
@@ -12911,7 +12917,7 @@
         <v>77</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>82</v>
@@ -12940,10 +12946,10 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -12969,10 +12975,10 @@
         <v>159</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="M99" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N99" s="2"/>
       <c r="O99" s="2"/>
@@ -13023,7 +13029,7 @@
         <v>77</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>82</v>
@@ -13038,7 +13044,7 @@
         <v>77</v>
       </c>
       <c r="AK99" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL99" t="s" s="2">
         <v>77</v>
@@ -13052,10 +13058,10 @@
     </row>
     <row r="100" hidden="true">
       <c r="A100" t="s" s="2">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -13084,7 +13090,7 @@
         <v>132</v>
       </c>
       <c r="M100" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N100" t="s" s="2">
         <v>134</v>
@@ -13137,7 +13143,7 @@
         <v>77</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>82</v>
@@ -13152,7 +13158,7 @@
         <v>136</v>
       </c>
       <c r="AK100" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL100" t="s" s="2">
         <v>77</v>
@@ -13166,14 +13172,14 @@
     </row>
     <row r="101" hidden="true">
       <c r="A101" t="s" s="2">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E101" s="2"/>
       <c r="F101" t="s" s="2">
@@ -13195,10 +13201,10 @@
         <v>131</v>
       </c>
       <c r="L101" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M101" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N101" t="s" s="2">
         <v>134</v>
@@ -13253,7 +13259,7 @@
         <v>77</v>
       </c>
       <c r="AF101" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>82</v>
@@ -13282,10 +13288,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -13311,10 +13317,10 @@
         <v>106</v>
       </c>
       <c r="L102" t="s" s="2">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="M102" t="s" s="2">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="N102" s="2"/>
       <c r="O102" s="2"/>
@@ -13365,7 +13371,7 @@
         <v>77</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>78</v>
@@ -13394,10 +13400,10 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -13423,10 +13429,10 @@
         <v>159</v>
       </c>
       <c r="L103" t="s" s="2">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="M103" t="s" s="2">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="N103" s="2"/>
       <c r="O103" s="2"/>
@@ -13477,7 +13483,7 @@
         <v>77</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>82</v>
@@ -13506,10 +13512,10 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -13535,10 +13541,10 @@
         <v>159</v>
       </c>
       <c r="L104" t="s" s="2">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="M104" t="s" s="2">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="N104" s="2"/>
       <c r="O104" s="2"/>
@@ -13589,7 +13595,7 @@
         <v>77</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>82</v>
@@ -13618,10 +13624,10 @@
     </row>
     <row r="105" hidden="true">
       <c r="A105" t="s" s="2">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -13644,19 +13650,19 @@
         <v>77</v>
       </c>
       <c r="K105" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L105" t="s" s="2">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="M105" t="s" s="2">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="N105" t="s" s="2">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O105" t="s" s="2">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="P105" t="s" s="2">
         <v>77</v>
@@ -13705,7 +13711,7 @@
         <v>77</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>82</v>
@@ -13734,10 +13740,10 @@
     </row>
     <row r="106" hidden="true">
       <c r="A106" t="s" s="2">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -13763,10 +13769,10 @@
         <v>159</v>
       </c>
       <c r="L106" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="M106" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N106" s="2"/>
       <c r="O106" s="2"/>
@@ -13817,7 +13823,7 @@
         <v>77</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>82</v>
@@ -13832,7 +13838,7 @@
         <v>77</v>
       </c>
       <c r="AK106" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL106" t="s" s="2">
         <v>77</v>
@@ -13846,10 +13852,10 @@
     </row>
     <row r="107" hidden="true">
       <c r="A107" t="s" s="2">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -13878,7 +13884,7 @@
         <v>132</v>
       </c>
       <c r="M107" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N107" t="s" s="2">
         <v>134</v>
@@ -13931,7 +13937,7 @@
         <v>77</v>
       </c>
       <c r="AF107" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="AG107" t="s" s="2">
         <v>82</v>
@@ -13946,7 +13952,7 @@
         <v>136</v>
       </c>
       <c r="AK107" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL107" t="s" s="2">
         <v>77</v>
@@ -13960,14 +13966,14 @@
     </row>
     <row r="108" hidden="true">
       <c r="A108" t="s" s="2">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E108" s="2"/>
       <c r="F108" t="s" s="2">
@@ -13989,10 +13995,10 @@
         <v>131</v>
       </c>
       <c r="L108" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M108" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N108" t="s" s="2">
         <v>134</v>
@@ -14047,7 +14053,7 @@
         <v>77</v>
       </c>
       <c r="AF108" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AG108" t="s" s="2">
         <v>82</v>
@@ -14076,10 +14082,10 @@
     </row>
     <row r="109" hidden="true">
       <c r="A109" t="s" s="2">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -14105,13 +14111,13 @@
         <v>106</v>
       </c>
       <c r="L109" t="s" s="2">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="M109" t="s" s="2">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="N109" t="s" s="2">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="O109" s="2"/>
       <c r="P109" t="s" s="2">
@@ -14161,7 +14167,7 @@
         <v>77</v>
       </c>
       <c r="AF109" t="s" s="2">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="AG109" t="s" s="2">
         <v>82</v>
@@ -14190,10 +14196,10 @@
     </row>
     <row r="110" hidden="true">
       <c r="A110" t="s" s="2">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -14216,16 +14222,16 @@
         <v>77</v>
       </c>
       <c r="K110" t="s" s="2">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="L110" t="s" s="2">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="M110" t="s" s="2">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="N110" t="s" s="2">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="O110" s="2"/>
       <c r="P110" t="s" s="2">
@@ -14251,13 +14257,13 @@
         <v>77</v>
       </c>
       <c r="X110" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="Y110" t="s" s="2">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="Z110" t="s" s="2">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="AA110" t="s" s="2">
         <v>77</v>
@@ -14275,7 +14281,7 @@
         <v>77</v>
       </c>
       <c r="AF110" t="s" s="2">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="AG110" t="s" s="2">
         <v>82</v>
@@ -14304,10 +14310,10 @@
     </row>
     <row r="111" hidden="true">
       <c r="A111" t="s" s="2">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
@@ -14333,10 +14339,10 @@
         <v>159</v>
       </c>
       <c r="L111" t="s" s="2">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="M111" t="s" s="2">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="N111" s="2"/>
       <c r="O111" s="2"/>
@@ -14387,7 +14393,7 @@
         <v>77</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>78</v>
@@ -14416,10 +14422,10 @@
     </row>
     <row r="112" hidden="true">
       <c r="A112" t="s" s="2">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -14442,13 +14448,13 @@
         <v>77</v>
       </c>
       <c r="K112" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L112" t="s" s="2">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="M112" t="s" s="2">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="N112" s="2"/>
       <c r="O112" s="2"/>
@@ -14499,7 +14505,7 @@
         <v>77</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="AG112" t="s" s="2">
         <v>82</v>
@@ -14528,10 +14534,10 @@
     </row>
     <row r="113" hidden="true">
       <c r="A113" t="s" s="2">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -14557,10 +14563,10 @@
         <v>159</v>
       </c>
       <c r="L113" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="M113" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="N113" s="2"/>
       <c r="O113" s="2"/>
@@ -14611,7 +14617,7 @@
         <v>77</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>82</v>
@@ -14626,7 +14632,7 @@
         <v>77</v>
       </c>
       <c r="AK113" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL113" t="s" s="2">
         <v>77</v>
@@ -14640,10 +14646,10 @@
     </row>
     <row r="114" hidden="true">
       <c r="A114" t="s" s="2">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -14672,7 +14678,7 @@
         <v>132</v>
       </c>
       <c r="M114" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N114" t="s" s="2">
         <v>134</v>
@@ -14725,7 +14731,7 @@
         <v>77</v>
       </c>
       <c r="AF114" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="AG114" t="s" s="2">
         <v>82</v>
@@ -14740,7 +14746,7 @@
         <v>136</v>
       </c>
       <c r="AK114" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AL114" t="s" s="2">
         <v>77</v>
@@ -14754,14 +14760,14 @@
     </row>
     <row r="115" hidden="true">
       <c r="A115" t="s" s="2">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E115" s="2"/>
       <c r="F115" t="s" s="2">
@@ -14783,10 +14789,10 @@
         <v>131</v>
       </c>
       <c r="L115" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M115" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N115" t="s" s="2">
         <v>134</v>
@@ -14841,7 +14847,7 @@
         <v>77</v>
       </c>
       <c r="AF115" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AG115" t="s" s="2">
         <v>82</v>
@@ -14870,10 +14876,10 @@
     </row>
     <row r="116" hidden="true">
       <c r="A116" t="s" s="2">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -14899,10 +14905,10 @@
         <v>106</v>
       </c>
       <c r="L116" t="s" s="2">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="M116" t="s" s="2">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="N116" s="2"/>
       <c r="O116" s="2"/>
@@ -14953,7 +14959,7 @@
         <v>77</v>
       </c>
       <c r="AF116" t="s" s="2">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="AG116" t="s" s="2">
         <v>78</v>
@@ -14982,10 +14988,10 @@
     </row>
     <row r="117" hidden="true">
       <c r="A117" t="s" s="2">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -15008,13 +15014,13 @@
         <v>77</v>
       </c>
       <c r="K117" t="s" s="2">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="L117" t="s" s="2">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="M117" t="s" s="2">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="N117" s="2"/>
       <c r="O117" s="2"/>
@@ -15065,7 +15071,7 @@
         <v>77</v>
       </c>
       <c r="AF117" t="s" s="2">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="AG117" t="s" s="2">
         <v>78</v>
@@ -15094,10 +15100,10 @@
     </row>
     <row r="118" hidden="true">
       <c r="A118" t="s" s="2">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" t="s" s="2">
@@ -15123,10 +15129,10 @@
         <v>79</v>
       </c>
       <c r="L118" t="s" s="2">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="M118" t="s" s="2">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="N118" s="2"/>
       <c r="O118" s="2"/>
@@ -15177,7 +15183,7 @@
         <v>77</v>
       </c>
       <c r="AF118" t="s" s="2">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="AG118" t="s" s="2">
         <v>82</v>

</xml_diff>